<commit_message>
Reworked examples to load profile events from worksheet if worksheet is set as the import method
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/environment/random/random_v4.xlsx
+++ b/src/rattlesnake/examples/environment/random/random_v4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples\environment\random\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B53E8EB-A9CC-42C3-B4C6-1672FF027C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97ADBCE0-5CB3-4EAB-BBD7-A37A0154036F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6260" yWindow="4890" windowWidth="28790" windowHeight="15350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6260" yWindow="4890" windowWidth="28790" windowHeight="15350" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Random 0" sheetId="3" r:id="rId1"/>
@@ -1036,6 +1036,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.08984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
User interface now loads system identification when loading from a Rattlesnake object. Fixed issues with Random Vibration profile event sending the wrong test level to the data collector during user interface profile event building.
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/environment/random/random_v4.xlsx
+++ b/src/rattlesnake/examples/environment/random/random_v4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples\environment\random\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97ADBCE0-5CB3-4EAB-BBD7-A37A0154036F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F583C4-54A1-4D8C-8A80-7A0983F815D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6260" yWindow="4890" windowWidth="28790" windowHeight="15350" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="96">
   <si>
     <t>Random 0</t>
   </si>
@@ -294,9 +294,6 @@
   </si>
   <si>
     <t>Save Control Data</t>
-  </si>
-  <si>
-    <t>18.0</t>
   </si>
   <si>
     <t>Change Specification</t>
@@ -1114,19 +1111,19 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>91</v>
+      <c r="A7">
+        <v>17</v>
       </c>
       <c r="B7" t="s">
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B8" t="s">
         <v>0</v>
@@ -1137,7 +1134,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B9" t="s">
         <v>0</v>
@@ -1148,24 +1145,24 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
         <v>81</v>
       </c>
       <c r="C10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
         <v>81</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added in filetype discovery for v3 netcdf files.
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/environment/random/random_v4.xlsx
+++ b/src/rattlesnake/examples/environment/random/random_v4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples\environment\random\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F583C4-54A1-4D8C-8A80-7A0983F815D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D94CA6-6275-4404-9665-306CDAB85527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6260" yWindow="4890" windowWidth="28790" windowHeight="15350" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Random 0" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="95">
   <si>
     <t>Random 0</t>
   </si>
@@ -243,9 +243,6 @@
   </si>
   <si>
     <t>Response Transformation Matrix:</t>
-  </si>
-  <si>
-    <t>None</t>
   </si>
   <si>
     <t>Output Transformation Matrix:</t>
@@ -648,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -1000,7 +997,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>71</v>
       </c>
@@ -1008,20 +1005,304 @@
         <v>72</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>73</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>75</v>
-      </c>
-      <c r="B35" t="s">
-        <v>74</v>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B39">
+        <v>0</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B40">
+        <v>0</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B41">
+        <v>0</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B42">
+        <v>0</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B43">
+        <v>0</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B44">
+        <v>0</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <v>1</v>
+      </c>
+      <c r="J44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B45">
+        <v>0</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1040,74 +1321,74 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" t="s">
         <v>76</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>77</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>78</v>
-      </c>
-      <c r="D1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
         <v>80</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>81</v>
-      </c>
-      <c r="C2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B3" t="s">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
         <v>84</v>
       </c>
-      <c r="B4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>85</v>
-      </c>
-      <c r="D4" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
         <v>87</v>
-      </c>
-      <c r="B5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
         <v>89</v>
-      </c>
-      <c r="B6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -1118,51 +1399,51 @@
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" t="s">
         <v>93</v>
-      </c>
-      <c r="B10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added percent lines out to random environment templates.
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/environment/random/random_v4.xlsx
+++ b/src/rattlesnake/examples/environment/random/random_v4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples\environment\random\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller\src\rattlesnake\examples\environment\random\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D94CA6-6275-4404-9665-306CDAB85527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D40B8C84-3E71-4352-BCE6-B81358A67279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="96">
   <si>
     <t>Random 0</t>
   </si>
@@ -306,6 +306,9 @@
   </si>
   <si>
     <t>Stop Hardware</t>
+  </si>
+  <si>
+    <t>Percent Lines Out</t>
   </si>
 </sst>
 </file>
@@ -645,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -760,271 +763,268 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>26</v>
+        <v>95</v>
+      </c>
+      <c r="B11">
+        <v>0.1</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15">
-        <v>2</v>
-      </c>
-      <c r="D15">
-        <v>3</v>
+        <v>32</v>
+      </c>
+      <c r="C15" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B16">
-        <v>5</v>
-      </c>
-      <c r="C16" t="s">
-        <v>36</v>
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B17">
-        <v>2048</v>
+        <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" t="s">
-        <v>40</v>
+        <v>37</v>
+      </c>
+      <c r="B18">
+        <v>2048</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19">
-        <v>20</v>
+        <v>39</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B20">
         <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B21">
-        <v>0.01</v>
+        <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>48</v>
-      </c>
-      <c r="B22" t="s">
-        <v>49</v>
+        <v>46</v>
+      </c>
+      <c r="B22">
+        <v>0.01</v>
       </c>
       <c r="C22" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23">
-        <v>0.01</v>
+        <v>48</v>
+      </c>
+      <c r="B23" t="s">
+        <v>49</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="C24" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B25">
-        <v>1024</v>
+        <v>0</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B26">
-        <v>0.5</v>
+        <v>1024</v>
       </c>
       <c r="C26" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>59</v>
-      </c>
-      <c r="B27" t="s">
-        <v>2</v>
+        <v>57</v>
+      </c>
+      <c r="B27">
+        <v>0.5</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B28" t="s">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29">
-        <v>50</v>
+        <v>61</v>
+      </c>
+      <c r="B29" t="s">
+        <v>21</v>
       </c>
       <c r="C29" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B30">
         <v>50</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B31">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B32">
         <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>71</v>
+        <v>69</v>
+      </c>
+      <c r="B33">
+        <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>73</v>
       </c>
-      <c r="B34">
+      <c r="B35">
         <v>1</v>
       </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-      <c r="D34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B35">
-        <v>0</v>
-      </c>
       <c r="C35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -1035,50 +1035,32 @@
         <v>0</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+      <c r="D37">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>74</v>
       </c>
-      <c r="B37">
+      <c r="B38">
         <v>1</v>
       </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
-      <c r="D37">
-        <v>0</v>
-      </c>
-      <c r="E37">
-        <v>0</v>
-      </c>
-      <c r="F37">
-        <v>0</v>
-      </c>
-      <c r="G37">
-        <v>0</v>
-      </c>
-      <c r="H37">
-        <v>0</v>
-      </c>
-      <c r="I37">
-        <v>0</v>
-      </c>
-      <c r="J37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B38">
-        <v>0</v>
-      </c>
       <c r="C38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38">
         <v>0</v>
@@ -1107,10 +1089,10 @@
         <v>0</v>
       </c>
       <c r="C39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E39">
         <v>0</v>
@@ -1139,10 +1121,10 @@
         <v>0</v>
       </c>
       <c r="D40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -1171,10 +1153,10 @@
         <v>0</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41">
         <v>0</v>
@@ -1203,10 +1185,10 @@
         <v>0</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H42">
         <v>0</v>
@@ -1235,10 +1217,10 @@
         <v>0</v>
       </c>
       <c r="G43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I43">
         <v>0</v>
@@ -1267,10 +1249,10 @@
         <v>0</v>
       </c>
       <c r="H44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J44">
         <v>0</v>
@@ -1299,9 +1281,38 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B46">
+        <v>0</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
+      </c>
+      <c r="I46">
+        <v>0</v>
+      </c>
+      <c r="J46">
         <v>1</v>
       </c>
     </row>

</xml_diff>